<commit_message>
update CIU EAAE considerando validaciones manuales
</commit_message>
<xml_diff>
--- a/data/analysis-data/20260528_panel_eaae.xlsx
+++ b/data/analysis-data/20260528_panel_eaae.xlsx
@@ -5,6 +5,8 @@
     <sheet name="eaae" sheetId="1" r:id="rId1"/>
     <sheet name="rama-C" sheetId="2" r:id="rId2"/>
     <sheet name="check-calidad-C" sheetId="3" r:id="rId3"/>
+    <sheet name="economia_total" sheetId="4" r:id="rId4"/>
+    <sheet name="check-calidad-total" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -2780,7 +2782,7 @@
         <v>13982311018.7924</v>
       </c>
       <c r="J42">
-        <v>63928.8527653802</v>
+        <v>63928</v>
       </c>
       <c r="K42">
         <v>6516136919.59274</v>
@@ -2908,7 +2910,7 @@
         <v>5922562988.59692</v>
       </c>
       <c r="J44">
-        <v>30494.2930531318</v>
+        <v>30494</v>
       </c>
       <c r="K44">
         <v>1469272662.01753</v>
@@ -2972,7 +2974,7 @@
         <v>7762570422.74903</v>
       </c>
       <c r="J45">
-        <v>24730.4372781752</v>
+        <v>24730</v>
       </c>
       <c r="K45">
         <v>8796636907.33007</v>
@@ -3100,7 +3102,7 @@
         <v>2384834809.22453</v>
       </c>
       <c r="J47">
-        <v>17724.6547481738</v>
+        <v>17724</v>
       </c>
       <c r="K47">
         <v>434412281.532599</v>
@@ -3164,7 +3166,7 @@
         <v>1281002871.44522</v>
       </c>
       <c r="J48">
-        <v>8781.4219114219</v>
+        <v>8781</v>
       </c>
       <c r="K48">
         <v>103429067.765734</v>
@@ -3228,7 +3230,7 @@
         <v>9970650180.39649</v>
       </c>
       <c r="J49">
-        <v>43328.3015802601</v>
+        <v>43328</v>
       </c>
       <c r="K49">
         <v>887370869.316838</v>
@@ -3292,7 +3294,7 @@
         <v>19975832217.4233</v>
       </c>
       <c r="J50">
-        <v>100576.012248596</v>
+        <v>100576</v>
       </c>
       <c r="K50">
         <v>17359289524.5189</v>
@@ -3420,7 +3422,7 @@
         <v>13444886138.7346</v>
       </c>
       <c r="J52">
-        <v>79220.2596892227</v>
+        <v>79220</v>
       </c>
       <c r="K52">
         <v>4100430982.73955</v>
@@ -3484,7 +3486,7 @@
         <v>12273618258.21</v>
       </c>
       <c r="J53">
-        <v>41934.0927895859</v>
+        <v>41934</v>
       </c>
       <c r="K53">
         <v>11396300915.6555</v>
@@ -3548,7 +3550,7 @@
         <v>2179920722.5</v>
       </c>
       <c r="J54">
-        <v>15648.6666666667</v>
+        <v>15648</v>
       </c>
       <c r="K54">
         <v>195801676.739444</v>
@@ -3612,7 +3614,7 @@
         <v>5021743121.0367</v>
       </c>
       <c r="J55">
-        <v>37538.4958383639</v>
+        <v>37538</v>
       </c>
       <c r="K55">
         <v>848226002.603641</v>
@@ -3676,7 +3678,7 @@
         <v>3247046965.36316</v>
       </c>
       <c r="J56">
-        <v>31985.5374078303</v>
+        <v>31985</v>
       </c>
       <c r="K56">
         <v>279363983.340499</v>
@@ -3740,7 +3742,7 @@
         <v>13976350426.3324</v>
       </c>
       <c r="J57">
-        <v>66667.8288745664</v>
+        <v>66667</v>
       </c>
       <c r="K57">
         <v>1096182660.40037</v>
@@ -3804,7 +3806,7 @@
         <v>145858508</v>
       </c>
       <c r="J58">
-        <v>868.2</v>
+        <v>868</v>
       </c>
       <c r="K58">
         <v>186931359</v>
@@ -3868,7 +3870,7 @@
         <v>24291156273.8742</v>
       </c>
       <c r="J59">
-        <v>103902.68580704</v>
+        <v>103902</v>
       </c>
       <c r="K59">
         <v>17442926160.2144</v>
@@ -3932,7 +3934,7 @@
         <v>5256625206.64255</v>
       </c>
       <c r="J60">
-        <v>11916.4763107917</v>
+        <v>11916</v>
       </c>
       <c r="K60">
         <v>3559653461.54619</v>
@@ -3996,7 +3998,7 @@
         <v>16738002803.4909</v>
       </c>
       <c r="J61">
-        <v>92823.4639331325</v>
+        <v>92823</v>
       </c>
       <c r="K61">
         <v>5221207956.50504</v>
@@ -4060,7 +4062,7 @@
         <v>17013000481.5745</v>
       </c>
       <c r="J62">
-        <v>51846.5635697458</v>
+        <v>51846</v>
       </c>
       <c r="K62">
         <v>13636148745.2706</v>
@@ -4124,7 +4126,7 @@
         <v>2634263481.44725</v>
       </c>
       <c r="J63">
-        <v>18496.7499281771</v>
+        <v>18496</v>
       </c>
       <c r="K63">
         <v>373654444.044741</v>
@@ -4188,7 +4190,7 @@
         <v>6100613117.15937</v>
       </c>
       <c r="J64">
-        <v>46616.4459379282</v>
+        <v>46616</v>
       </c>
       <c r="K64">
         <v>777880193.465546</v>
@@ -4252,7 +4254,7 @@
         <v>3566664247.15113</v>
       </c>
       <c r="J65">
-        <v>31795.1355979198</v>
+        <v>31795</v>
       </c>
       <c r="K65">
         <v>246447048.810283</v>
@@ -4316,7 +4318,7 @@
         <v>16994715654.6684</v>
       </c>
       <c r="J66">
-        <v>69259.1383535502</v>
+        <v>69259</v>
       </c>
       <c r="K66">
         <v>1612498764.51498</v>
@@ -4380,7 +4382,7 @@
         <v>1475484549.7381</v>
       </c>
       <c r="J67">
-        <v>8919.44444444445</v>
+        <v>8919</v>
       </c>
       <c r="K67">
         <v>252867504.079365</v>
@@ -4444,7 +4446,7 @@
         <v>29743370612.9925</v>
       </c>
       <c r="J68">
-        <v>104036.647790835</v>
+        <v>104036</v>
       </c>
       <c r="K68">
         <v>7961085386.42427</v>
@@ -4508,7 +4510,7 @@
         <v>6068798136.1</v>
       </c>
       <c r="J69">
-        <v>12290.2</v>
+        <v>12290</v>
       </c>
       <c r="K69">
         <v>4760493305.9</v>
@@ -4572,7 +4574,7 @@
         <v>21123382960.9343</v>
       </c>
       <c r="J70">
-        <v>99621.6072677287</v>
+        <v>99621</v>
       </c>
       <c r="K70">
         <v>6918031617.39357</v>
@@ -4636,7 +4638,7 @@
         <v>20593240105.1192</v>
       </c>
       <c r="J71">
-        <v>54292.7354939143</v>
+        <v>54292</v>
       </c>
       <c r="K71">
         <v>13488357170.3188</v>
@@ -4700,7 +4702,7 @@
         <v>2965205187.34601</v>
       </c>
       <c r="J72">
-        <v>17697.4711439328</v>
+        <v>17697</v>
       </c>
       <c r="K72">
         <v>780365867.979899</v>
@@ -4764,7 +4766,7 @@
         <v>9817803133.81814</v>
       </c>
       <c r="J73">
-        <v>61772.2605977847</v>
+        <v>61772</v>
       </c>
       <c r="K73">
         <v>1092830465.86284</v>
@@ -4828,7 +4830,7 @@
         <v>4330630889.86295</v>
       </c>
       <c r="J74">
-        <v>30152.8270148521</v>
+        <v>30152</v>
       </c>
       <c r="K74">
         <v>396857073.372038</v>
@@ -4892,7 +4894,7 @@
         <v>19081212214.0546</v>
       </c>
       <c r="J75">
-        <v>74044.7710593574</v>
+        <v>74044</v>
       </c>
       <c r="K75">
         <v>1722104161.79037</v>
@@ -4956,7 +4958,7 @@
         <v>3385269866.45843</v>
       </c>
       <c r="J76">
-        <v>23552.4923506787</v>
+        <v>23552</v>
       </c>
       <c r="K76">
         <v>375209335.057403</v>
@@ -5020,7 +5022,7 @@
         <v>34131850283.3496</v>
       </c>
       <c r="J77">
-        <v>112274.193929867</v>
+        <v>112274</v>
       </c>
       <c r="K77">
         <v>10581328732.3151</v>
@@ -5084,7 +5086,7 @@
         <v>7026644454</v>
       </c>
       <c r="J78">
-        <v>12607.25</v>
+        <v>12607</v>
       </c>
       <c r="K78">
         <v>9171112853</v>
@@ -5148,7 +5150,7 @@
         <v>26747076212.0739</v>
       </c>
       <c r="J79">
-        <v>112666.908623568</v>
+        <v>112666</v>
       </c>
       <c r="K79">
         <v>8076935906.25148</v>
@@ -5212,7 +5214,7 @@
         <v>24322396293.5033</v>
       </c>
       <c r="J80">
-        <v>59920.0134664369</v>
+        <v>59920</v>
       </c>
       <c r="K80">
         <v>15474182798.7012</v>
@@ -5276,7 +5278,7 @@
         <v>4544184703.87225</v>
       </c>
       <c r="J81">
-        <v>24412.3920054842</v>
+        <v>24412</v>
       </c>
       <c r="K81">
         <v>2294878556.65625</v>
@@ -5340,7 +5342,7 @@
         <v>15123683950.9074</v>
       </c>
       <c r="J82">
-        <v>73624.3306332459</v>
+        <v>73624</v>
       </c>
       <c r="K82">
         <v>1864415627.99804</v>
@@ -5404,7 +5406,7 @@
         <v>5107759058.78456</v>
       </c>
       <c r="J83">
-        <v>31457.153758589</v>
+        <v>31457</v>
       </c>
       <c r="K83">
         <v>473420936.084401</v>
@@ -5468,7 +5470,7 @@
         <v>23647226705.2188</v>
       </c>
       <c r="J84">
-        <v>75954.1198662344</v>
+        <v>75954</v>
       </c>
       <c r="K84">
         <v>12635303080.9613</v>
@@ -5532,7 +5534,7 @@
         <v>4034922088.96297</v>
       </c>
       <c r="J85">
-        <v>19366.4060191436</v>
+        <v>19366</v>
       </c>
       <c r="K85">
         <v>505220495.584963</v>
@@ -5596,7 +5598,7 @@
         <v>38240756792.5859</v>
       </c>
       <c r="J86">
-        <v>109399.623065035</v>
+        <v>109399</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
@@ -5666,7 +5668,7 @@
         <v>7835641471.58971</v>
       </c>
       <c r="J87">
-        <v>14529.5853293553</v>
+        <v>14529</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -5736,7 +5738,7 @@
         <v>31869388118.3108</v>
       </c>
       <c r="J88">
-        <v>114837.617814199</v>
+        <v>114837</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -5806,7 +5808,7 @@
         <v>35431447242.5919</v>
       </c>
       <c r="J89">
-        <v>74688.4488608632</v>
+        <v>74688</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -5876,7 +5878,7 @@
         <v>3667389791.61286</v>
       </c>
       <c r="J90">
-        <v>20434.2780410222</v>
+        <v>20434</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -5946,7 +5948,7 @@
         <v>16480028160.395</v>
       </c>
       <c r="J91">
-        <v>74963.7941177931</v>
+        <v>74963</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -6016,7 +6018,7 @@
         <v>6349584271.71878</v>
       </c>
       <c r="J92">
-        <v>32998.5544077656</v>
+        <v>32998</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -6086,7 +6088,7 @@
         <v>27717309591.7406</v>
       </c>
       <c r="J93">
-        <v>79386.7887610837</v>
+        <v>79386</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -6156,7 +6158,7 @@
         <v>5379043920.79628</v>
       </c>
       <c r="J94">
-        <v>21219.0796480612</v>
+        <v>21219</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -6226,7 +6228,7 @@
         <v>352142647.759346</v>
       </c>
       <c r="J95">
-        <v>1006.67903528926</v>
+        <v>1006</v>
       </c>
       <c r="K95">
         <v>300655513.741754</v>
@@ -6290,7 +6292,7 @@
         <v>43787874689.4251</v>
       </c>
       <c r="J96">
-        <v>110138.749533575</v>
+        <v>110138</v>
       </c>
       <c r="K96">
         <v>17144628448.139</v>
@@ -6354,7 +6356,7 @@
         <v>9907071211.93849</v>
       </c>
       <c r="J97">
-        <v>15343.035964684</v>
+        <v>15343</v>
       </c>
       <c r="K97">
         <v>8642302809.39199</v>
@@ -6418,7 +6420,7 @@
         <v>39444683778.099</v>
       </c>
       <c r="J98">
-        <v>122466.610158149</v>
+        <v>122466</v>
       </c>
       <c r="K98">
         <v>16208013394.8697</v>
@@ -6482,7 +6484,7 @@
         <v>33818979819.7855</v>
       </c>
       <c r="J99">
-        <v>67775.4773051096</v>
+        <v>67775</v>
       </c>
       <c r="K99">
         <v>16856230160.9046</v>
@@ -6546,7 +6548,7 @@
         <v>4351816270.32081</v>
       </c>
       <c r="J100">
-        <v>21646.754350659</v>
+        <v>21646</v>
       </c>
       <c r="K100">
         <v>1538388122.94021</v>
@@ -6610,7 +6612,7 @@
         <v>6882689620.71421</v>
       </c>
       <c r="J101">
-        <v>9841.91104546465</v>
+        <v>9841</v>
       </c>
       <c r="K101">
         <v>416105780.322707</v>
@@ -6674,7 +6676,7 @@
         <v>19261904119.4494</v>
       </c>
       <c r="J102">
-        <v>79318.368872498</v>
+        <v>79318</v>
       </c>
       <c r="K102">
         <v>5100184630.97153</v>
@@ -6738,7 +6740,7 @@
         <v>7576950185.61996</v>
       </c>
       <c r="J103">
-        <v>34814.3843234316</v>
+        <v>34814</v>
       </c>
       <c r="K103">
         <v>587838087.3527</v>
@@ -6802,7 +6804,7 @@
         <v>32753414485.3581</v>
       </c>
       <c r="J104">
-        <v>81498.5538251129</v>
+        <v>81498</v>
       </c>
       <c r="K104">
         <v>2517220413.0552</v>
@@ -6866,7 +6868,7 @@
         <v>6242340781.29273</v>
       </c>
       <c r="J105">
-        <v>20993.2727975595</v>
+        <v>20993</v>
       </c>
       <c r="K105">
         <v>1091009522.15292</v>
@@ -6930,7 +6932,7 @@
         <v>418975808.350729</v>
       </c>
       <c r="J106">
-        <v>1107.28968018305</v>
+        <v>1107</v>
       </c>
       <c r="K106">
         <v>433254714.012333</v>
@@ -6994,7 +6996,7 @@
         <v>50186679222.5088</v>
       </c>
       <c r="J107">
-        <v>109797.749814658</v>
+        <v>109797</v>
       </c>
       <c r="K107">
         <v>28790672811.2985</v>
@@ -7058,7 +7060,7 @@
         <v>11156680423.1465</v>
       </c>
       <c r="J108">
-        <v>15449.1998868569</v>
+        <v>15449</v>
       </c>
       <c r="K108">
         <v>9792573764.66106</v>
@@ -7122,7 +7124,7 @@
         <v>47556638703.632</v>
       </c>
       <c r="J109">
-        <v>129905.885876198</v>
+        <v>129905</v>
       </c>
       <c r="K109">
         <v>15431546310.898</v>
@@ -7186,7 +7188,7 @@
         <v>40907826937.4688</v>
       </c>
       <c r="J110">
-        <v>74603.9951949249</v>
+        <v>74603</v>
       </c>
       <c r="K110">
         <v>30338349956.5551</v>
@@ -7250,7 +7252,7 @@
         <v>5097565016.30734</v>
       </c>
       <c r="J111">
-        <v>23477.8944130387</v>
+        <v>23477</v>
       </c>
       <c r="K111">
         <v>1212981784.36202</v>
@@ -7314,7 +7316,7 @@
         <v>6198366275.33083</v>
       </c>
       <c r="J112">
-        <v>8995.69189572079</v>
+        <v>8995</v>
       </c>
       <c r="K112">
         <v>486641459.452508</v>
@@ -7378,7 +7380,7 @@
         <v>22855256399.2435</v>
       </c>
       <c r="J113">
-        <v>81735.9428957009</v>
+        <v>81735</v>
       </c>
       <c r="K113">
         <v>3447840611.69093</v>
@@ -7442,7 +7444,7 @@
         <v>9482672821.25763</v>
       </c>
       <c r="J114">
-        <v>40057.3910166575</v>
+        <v>40057</v>
       </c>
       <c r="K114">
         <v>558251499.614631</v>
@@ -7506,7 +7508,7 @@
         <v>38369574505.0875</v>
       </c>
       <c r="J115">
-        <v>83566.5934527804</v>
+        <v>83566</v>
       </c>
       <c r="K115">
         <v>3459232323.64235</v>
@@ -7570,7 +7572,7 @@
         <v>7487086853.33496</v>
       </c>
       <c r="J116">
-        <v>23601.5738369182</v>
+        <v>23601</v>
       </c>
       <c r="K116">
         <v>1680914697.25276</v>
@@ -7634,7 +7636,7 @@
         <v>515645948.601414</v>
       </c>
       <c r="J117">
-        <v>1116.80485864993</v>
+        <v>1116</v>
       </c>
       <c r="K117">
         <v>258656796.446423</v>
@@ -7698,7 +7700,7 @@
         <v>56837646365.6924</v>
       </c>
       <c r="J118">
-        <v>107700.426949954</v>
+        <v>107700</v>
       </c>
       <c r="K118">
         <v>78176629453.8231</v>
@@ -7762,7 +7764,7 @@
         <v>12417609182.1087</v>
       </c>
       <c r="J119">
-        <v>15772.3855100279</v>
+        <v>15772</v>
       </c>
       <c r="K119">
         <v>20692528407.245</v>
@@ -7826,7 +7828,7 @@
         <v>56309853657.2369</v>
       </c>
       <c r="J120">
-        <v>133998.565319341</v>
+        <v>133998</v>
       </c>
       <c r="K120">
         <v>15707268357.6361</v>
@@ -7890,7 +7892,7 @@
         <v>48451679069.9894</v>
       </c>
       <c r="J121">
-        <v>79518.9732275915</v>
+        <v>79518</v>
       </c>
       <c r="K121">
         <v>33656910135.3043</v>
@@ -7954,7 +7956,7 @@
         <v>5958119151.52059</v>
       </c>
       <c r="J122">
-        <v>24672.1867012927</v>
+        <v>24672</v>
       </c>
       <c r="K122">
         <v>469669407.46863</v>
@@ -8018,7 +8020,7 @@
         <v>8024572493.34533</v>
       </c>
       <c r="J123">
-        <v>10324.7429353487</v>
+        <v>10324</v>
       </c>
       <c r="K123">
         <v>581411007.741496</v>
@@ -8082,7 +8084,7 @@
         <v>27360957939.2389</v>
       </c>
       <c r="J124">
-        <v>88280.1168110962</v>
+        <v>88280</v>
       </c>
       <c r="K124">
         <v>3350964231.87533</v>
@@ -8146,7 +8148,7 @@
         <v>11416645625.0283</v>
       </c>
       <c r="J125">
-        <v>42075.7186398752</v>
+        <v>42075</v>
       </c>
       <c r="K125">
         <v>1660014143.06569</v>
@@ -8210,7 +8212,7 @@
         <v>44683724646.3054</v>
       </c>
       <c r="J126">
-        <v>88178.334111498</v>
+        <v>88178</v>
       </c>
       <c r="K126">
         <v>2965754005.78414</v>
@@ -8274,7 +8276,7 @@
         <v>8950181584.13468</v>
       </c>
       <c r="J127">
-        <v>25221.0912492698</v>
+        <v>25221</v>
       </c>
       <c r="K127">
         <v>1708167802.60063</v>
@@ -8338,7 +8340,7 @@
         <v>561211583.073811</v>
       </c>
       <c r="J128">
-        <v>1137.11496246499</v>
+        <v>1137</v>
       </c>
       <c r="K128">
         <v>252197995.586458</v>
@@ -8402,7 +8404,7 @@
         <v>61103872632.9691</v>
       </c>
       <c r="J129">
-        <v>103791.208900956</v>
+        <v>103791</v>
       </c>
       <c r="K129">
         <v>26806672376.5168</v>
@@ -8466,7 +8468,7 @@
         <v>14205432688.972</v>
       </c>
       <c r="J130">
-        <v>16253.8758929709</v>
+        <v>16253</v>
       </c>
       <c r="K130">
         <v>18195872414.6954</v>
@@ -8530,7 +8532,7 @@
         <v>67373300663.5271</v>
       </c>
       <c r="J131">
-        <v>136613.68561472</v>
+        <v>136613</v>
       </c>
       <c r="K131">
         <v>19503083471.2755</v>
@@ -8594,7 +8596,7 @@
         <v>53342737578.6859</v>
       </c>
       <c r="J132">
-        <v>77928.6306974964</v>
+        <v>77928</v>
       </c>
       <c r="K132">
         <v>23957271517.9884</v>
@@ -8658,7 +8660,7 @@
         <v>7055016645.92952</v>
       </c>
       <c r="J133">
-        <v>26120.1630855247</v>
+        <v>26120</v>
       </c>
       <c r="K133">
         <v>917162106.248329</v>
@@ -8722,7 +8724,7 @@
         <v>9636283095.24866</v>
       </c>
       <c r="J134">
-        <v>8615.02543064335</v>
+        <v>8615</v>
       </c>
       <c r="K134">
         <v>860505852.153555</v>
@@ -8786,7 +8788,7 @@
         <v>31307189934.06</v>
       </c>
       <c r="J135">
-        <v>87409.7828025273</v>
+        <v>87409</v>
       </c>
       <c r="K135">
         <v>4463144698.16174</v>
@@ -8850,7 +8852,7 @@
         <v>12653250965.7407</v>
       </c>
       <c r="J136">
-        <v>43320.9588139442</v>
+        <v>43320</v>
       </c>
       <c r="K136">
         <v>1254056387.89072</v>
@@ -8914,7 +8916,7 @@
         <v>49738341859.0136</v>
       </c>
       <c r="J137">
-        <v>91004.743757116</v>
+        <v>91004</v>
       </c>
       <c r="K137">
         <v>4205541725.55819</v>
@@ -8978,7 +8980,7 @@
         <v>11103337809.7628</v>
       </c>
       <c r="J138">
-        <v>26784.7444140958</v>
+        <v>26784</v>
       </c>
       <c r="K138">
         <v>4809343819.49825</v>
@@ -9042,7 +9044,7 @@
         <v>615830080.234561</v>
       </c>
       <c r="J139">
-        <v>1073.88621012172</v>
+        <v>1073</v>
       </c>
       <c r="K139">
         <v>297533326.572692</v>
@@ -9106,7 +9108,7 @@
         <v>65854041864.7401</v>
       </c>
       <c r="J140">
-        <v>100240.446716766</v>
+        <v>100240</v>
       </c>
       <c r="K140">
         <v>17409371770.145</v>
@@ -9170,7 +9172,7 @@
         <v>15147042266.5617</v>
       </c>
       <c r="J141">
-        <v>15985.0554961166</v>
+        <v>15985</v>
       </c>
       <c r="K141">
         <v>24220732119.0121</v>
@@ -9234,7 +9236,7 @@
         <v>74673824222.05</v>
       </c>
       <c r="J142">
-        <v>134970.232881947</v>
+        <v>134970</v>
       </c>
       <c r="K142">
         <v>19039502279.5032</v>
@@ -9298,7 +9300,7 @@
         <v>59143773552.2334</v>
       </c>
       <c r="J143">
-        <v>77002.7211578009</v>
+        <v>77002</v>
       </c>
       <c r="K143">
         <v>30975507900.4703</v>
@@ -9362,7 +9364,7 @@
         <v>7892244161.90428</v>
       </c>
       <c r="J144">
-        <v>27387.9632274893</v>
+        <v>27387</v>
       </c>
       <c r="K144">
         <v>1327194075.01277</v>
@@ -9426,7 +9428,7 @@
         <v>9749037723.33426</v>
       </c>
       <c r="J145">
-        <v>8845.49459970579</v>
+        <v>8845</v>
       </c>
       <c r="K145">
         <v>473648198.96946</v>
@@ -9490,7 +9492,7 @@
         <v>35008412528.6165</v>
       </c>
       <c r="J146">
-        <v>85150.636508229</v>
+        <v>85150</v>
       </c>
       <c r="K146">
         <v>3198246459.51799</v>
@@ -9554,7 +9556,7 @@
         <v>13868531293.0859</v>
       </c>
       <c r="J147">
-        <v>43488.7056430112</v>
+        <v>43488</v>
       </c>
       <c r="K147">
         <v>1043195455.97597</v>
@@ -9618,7 +9620,7 @@
         <v>56736304250.6962</v>
       </c>
       <c r="J148">
-        <v>94195.3478135749</v>
+        <v>94195</v>
       </c>
       <c r="K148">
         <v>4217551565.98928</v>
@@ -9682,7 +9684,7 @@
         <v>12248599787.3957</v>
       </c>
       <c r="J149">
-        <v>26143.6030298825</v>
+        <v>26143</v>
       </c>
       <c r="K149">
         <v>1781886760.90299</v>
@@ -9742,7 +9744,7 @@
         <v>657498303.126476</v>
       </c>
       <c r="J150">
-        <v>1143.14648326107</v>
+        <v>1143</v>
       </c>
       <c r="K150">
         <v>178531834.12</v>
@@ -9802,7 +9804,7 @@
         <v>70584977309.7717</v>
       </c>
       <c r="J151">
-        <v>97466.9972261083</v>
+        <v>97466</v>
       </c>
       <c r="K151">
         <v>17036239960.98</v>
@@ -9862,7 +9864,7 @@
         <v>16345164422.6205</v>
       </c>
       <c r="J152">
-        <v>15655.4570794662</v>
+        <v>15655</v>
       </c>
       <c r="K152">
         <v>17280534586.11</v>
@@ -9922,7 +9924,7 @@
         <v>83773687021.4621</v>
       </c>
       <c r="J153">
-        <v>135656.632398341</v>
+        <v>135656</v>
       </c>
       <c r="K153">
         <v>13617990498.48</v>
@@ -9982,7 +9984,7 @@
         <v>62823399111.9484</v>
       </c>
       <c r="J154">
-        <v>78171.6180235322</v>
+        <v>78171</v>
       </c>
       <c r="K154">
         <v>34929783219.94</v>
@@ -10042,7 +10044,7 @@
         <v>9679394384.86377</v>
       </c>
       <c r="J155">
-        <v>28334.960915636</v>
+        <v>28334</v>
       </c>
       <c r="K155">
         <v>1311167251.04</v>
@@ -10102,7 +10104,7 @@
         <v>10813488957.756</v>
       </c>
       <c r="J156">
-        <v>8876.39995075483</v>
+        <v>8876</v>
       </c>
       <c r="K156">
         <v>632101869.33</v>
@@ -10162,7 +10164,7 @@
         <v>39273088032.7173</v>
       </c>
       <c r="J157">
-        <v>84938.5654026166</v>
+        <v>84938</v>
       </c>
       <c r="K157">
         <v>3719661805.39</v>
@@ -10222,7 +10224,7 @@
         <v>15338221633.304</v>
       </c>
       <c r="J158">
-        <v>45842.6299277274</v>
+        <v>45842</v>
       </c>
       <c r="K158">
         <v>1488653768.45</v>
@@ -10282,7 +10284,7 @@
         <v>62279557165.4252</v>
       </c>
       <c r="J159">
-        <v>95779.2569705255</v>
+        <v>95779</v>
       </c>
       <c r="K159">
         <v>3802581537.55</v>
@@ -10342,7 +10344,7 @@
         <v>13563405187.742</v>
       </c>
       <c r="J160">
-        <v>27960.5373515114</v>
+        <v>27960</v>
       </c>
       <c r="K160">
         <v>1579242470.6</v>
@@ -10402,7 +10404,7 @@
         <v>739697413.948032</v>
       </c>
       <c r="J161">
-        <v>994.929780501368</v>
+        <v>994</v>
       </c>
       <c r="K161">
         <v>196164457.832162</v>
@@ -10462,7 +10464,7 @@
         <v>76120684622.3108</v>
       </c>
       <c r="J162">
-        <v>94566.085657076</v>
+        <v>94566</v>
       </c>
       <c r="K162">
         <v>21403883661.2124</v>
@@ -10522,7 +10524,7 @@
         <v>17126252016.251</v>
       </c>
       <c r="J163">
-        <v>15095.8252293306</v>
+        <v>15095</v>
       </c>
       <c r="K163">
         <v>12577353191.5351</v>
@@ -10582,7 +10584,7 @@
         <v>90901249122.1436</v>
       </c>
       <c r="J164">
-        <v>135287.458560132</v>
+        <v>135287</v>
       </c>
       <c r="K164">
         <v>16089418083.824</v>
@@ -10642,7 +10644,7 @@
         <v>69742900315.8983</v>
       </c>
       <c r="J165">
-        <v>77745.2715333279</v>
+        <v>77745</v>
       </c>
       <c r="K165">
         <v>34577901253.8122</v>
@@ -10702,7 +10704,7 @@
         <v>10137105272.648</v>
       </c>
       <c r="J166">
-        <v>27110.6388468626</v>
+        <v>27110</v>
       </c>
       <c r="K166">
         <v>1628004653.12449</v>
@@ -10762,7 +10764,7 @@
         <v>12016441095.1521</v>
       </c>
       <c r="J167">
-        <v>8436.61856220838</v>
+        <v>8436</v>
       </c>
       <c r="K167">
         <v>351799066.412128</v>
@@ -10822,7 +10824,7 @@
         <v>42724707255.2939</v>
       </c>
       <c r="J168">
-        <v>86112.0483831525</v>
+        <v>86112</v>
       </c>
       <c r="K168">
         <v>4057917354.12228</v>
@@ -10882,7 +10884,7 @@
         <v>17590784305.781</v>
       </c>
       <c r="J169">
-        <v>47307.3722095728</v>
+        <v>47307</v>
       </c>
       <c r="K169">
         <v>1115750373.55401</v>
@@ -10942,7 +10944,7 @@
         <v>71221189632.3407</v>
       </c>
       <c r="J170">
-        <v>99178.2772869773</v>
+        <v>99178</v>
       </c>
       <c r="K170">
         <v>3724177260.51046</v>
@@ -11002,7 +11004,7 @@
         <v>14269424366.2955</v>
       </c>
       <c r="J171">
-        <v>28259.1698447474</v>
+        <v>28259</v>
       </c>
       <c r="K171">
         <v>1915840614.7508</v>
@@ -11722,7 +11724,7 @@
         <v>740604801.387926</v>
       </c>
       <c r="J183">
-        <v>886.035890422914</v>
+        <v>886</v>
       </c>
       <c r="K183">
         <v>387600431.252534</v>
@@ -11782,7 +11784,7 @@
         <v>78278216489.3034</v>
       </c>
       <c r="J184">
-        <v>84764.4647407208</v>
+        <v>84764</v>
       </c>
       <c r="K184">
         <v>40941559983.9069</v>
@@ -11842,7 +11844,7 @@
         <v>19244127478.6691</v>
       </c>
       <c r="J185">
-        <v>14595.190706808</v>
+        <v>14595</v>
       </c>
       <c r="K185">
         <v>14080786427.6507</v>
@@ -11902,7 +11904,7 @@
         <v>95988303066.6241</v>
       </c>
       <c r="J186">
-        <v>127799.594136732</v>
+        <v>127799</v>
       </c>
       <c r="K186">
         <v>18619182864.6824</v>
@@ -11962,7 +11964,7 @@
         <v>69614073776.4868</v>
       </c>
       <c r="J187">
-        <v>65989.5521432639</v>
+        <v>65989</v>
       </c>
       <c r="K187">
         <v>22737288177.439</v>
@@ -12022,7 +12024,7 @@
         <v>6232911619.30963</v>
       </c>
       <c r="J188">
-        <v>16992.0677827898</v>
+        <v>16992</v>
       </c>
       <c r="K188">
         <v>1236378090.29549</v>
@@ -12082,7 +12084,7 @@
         <v>12512124636.3721</v>
       </c>
       <c r="J189">
-        <v>7516.43557715413</v>
+        <v>7516</v>
       </c>
       <c r="K189">
         <v>760413938.922126</v>
@@ -12142,7 +12144,7 @@
         <v>48979845822.5439</v>
       </c>
       <c r="J190">
-        <v>84506.3390107698</v>
+        <v>84506</v>
       </c>
       <c r="K190">
         <v>10182011019.1536</v>
@@ -12202,7 +12204,7 @@
         <v>18145753020.7882</v>
       </c>
       <c r="J191">
-        <v>43648.6160636176</v>
+        <v>43648</v>
       </c>
       <c r="K191">
         <v>1291629563.00379</v>
@@ -12262,7 +12264,7 @@
         <v>81808060721.763</v>
       </c>
       <c r="J192">
-        <v>98293.2131016928</v>
+        <v>98293</v>
       </c>
       <c r="K192">
         <v>4583337908.53789</v>
@@ -12322,7 +12324,7 @@
         <v>14224516464.7482</v>
       </c>
       <c r="J193">
-        <v>25255.6460799333</v>
+        <v>25255</v>
       </c>
       <c r="K193">
         <v>2148406210.29189</v>
@@ -12382,7 +12384,7 @@
         <v>942639331.341875</v>
       </c>
       <c r="J194">
-        <v>1221.27703280326</v>
+        <v>1221</v>
       </c>
       <c r="K194">
         <v>535413296.066923</v>
@@ -12442,7 +12444,7 @@
         <v>84122098877.8656</v>
       </c>
       <c r="J195">
-        <v>86333.0943782653</v>
+        <v>86333</v>
       </c>
       <c r="K195">
         <v>83942983585.5647</v>
@@ -12502,7 +12504,7 @@
         <v>20221632008.4409</v>
       </c>
       <c r="J196">
-        <v>14128.9637201459</v>
+        <v>14128</v>
       </c>
       <c r="K196">
         <v>15097593386.138</v>
@@ -12562,7 +12564,7 @@
         <v>95155129416.3319</v>
       </c>
       <c r="J197">
-        <v>131187.678965903</v>
+        <v>131187</v>
       </c>
       <c r="K197">
         <v>32633273093.592</v>
@@ -12622,7 +12624,7 @@
         <v>68176469340.4815</v>
       </c>
       <c r="J198">
-        <v>66121.0482403959</v>
+        <v>66121</v>
       </c>
       <c r="K198">
         <v>31816613640.5214</v>
@@ -12682,7 +12684,7 @@
         <v>7079050388.14224</v>
       </c>
       <c r="J199">
-        <v>22527.1368497778</v>
+        <v>22527</v>
       </c>
       <c r="K199">
         <v>3177150585.37297</v>
@@ -12742,7 +12744,7 @@
         <v>15423416558.2085</v>
       </c>
       <c r="J200">
-        <v>9729.03066197288</v>
+        <v>9729</v>
       </c>
       <c r="K200">
         <v>1098288138.06267</v>
@@ -12802,7 +12804,7 @@
         <v>59414119118.0736</v>
       </c>
       <c r="J201">
-        <v>98975.6115960444</v>
+        <v>98975</v>
       </c>
       <c r="K201">
         <v>10121111282.6722</v>
@@ -12862,7 +12864,7 @@
         <v>20472823337.4853</v>
       </c>
       <c r="J202">
-        <v>46075.3892527884</v>
+        <v>46075</v>
       </c>
       <c r="K202">
         <v>1462932383.7338</v>
@@ -12922,7 +12924,7 @@
         <v>84893592451.3226</v>
       </c>
       <c r="J203">
-        <v>101572.118517785</v>
+        <v>101572</v>
       </c>
       <c r="K203">
         <v>5379104877.85428</v>
@@ -12982,7 +12984,7 @@
         <v>14298850361.4134</v>
       </c>
       <c r="J204">
-        <v>25103.5732873284</v>
+        <v>25103</v>
       </c>
       <c r="K204">
         <v>2057069656.38168</v>
@@ -13042,7 +13044,7 @@
         <v>1077136328.27884</v>
       </c>
       <c r="J205">
-        <v>1379.56000823748</v>
+        <v>1379</v>
       </c>
       <c r="K205">
         <v>347532015.953246</v>
@@ -13102,7 +13104,7 @@
         <v>95609914033.8778</v>
       </c>
       <c r="J206">
-        <v>89467.5060887856</v>
+        <v>89467</v>
       </c>
       <c r="K206">
         <v>69687013752.2493</v>
@@ -13162,7 +13164,7 @@
         <v>20626352086.312</v>
       </c>
       <c r="J207">
-        <v>13915.1952344857</v>
+        <v>13915</v>
       </c>
       <c r="K207">
         <v>17801987415.9956</v>
@@ -13222,7 +13224,7 @@
         <v>106441380612.163</v>
       </c>
       <c r="J208">
-        <v>135877.300330261</v>
+        <v>135877</v>
       </c>
       <c r="K208">
         <v>25582362175.1944</v>
@@ -13282,7 +13284,7 @@
         <v>87162885551.2367</v>
       </c>
       <c r="J209">
-        <v>74447.36207913</v>
+        <v>74447</v>
       </c>
       <c r="K209">
         <v>41666501508.594</v>
@@ -13342,7 +13344,7 @@
         <v>9721139537.18689</v>
       </c>
       <c r="J210">
-        <v>25190.6652338519</v>
+        <v>25190</v>
       </c>
       <c r="K210">
         <v>2442655156.00974</v>
@@ -13402,7 +13404,7 @@
         <v>13563253468.8588</v>
       </c>
       <c r="J211">
-        <v>7781.15101445186</v>
+        <v>7781</v>
       </c>
       <c r="K211">
         <v>1211488493.10716</v>
@@ -13462,7 +13464,7 @@
         <v>65915211622.238</v>
       </c>
       <c r="J212">
-        <v>106629.01524402</v>
+        <v>106629</v>
       </c>
       <c r="K212">
         <v>9327884423.71499</v>
@@ -13522,7 +13524,7 @@
         <v>22170454088.5541</v>
       </c>
       <c r="J213">
-        <v>48186.0124638178</v>
+        <v>48186</v>
       </c>
       <c r="K213">
         <v>2031278865.74084</v>
@@ -13582,7 +13584,7 @@
         <v>84407646158.2658</v>
       </c>
       <c r="J214">
-        <v>97322.2928322129</v>
+        <v>97322</v>
       </c>
       <c r="K214">
         <v>5001096201.65267</v>
@@ -13642,7 +13644,7 @@
         <v>15559291269.3462</v>
       </c>
       <c r="J215">
-        <v>26889.283055257</v>
+        <v>26889</v>
       </c>
       <c r="K215">
         <v>7933531623.973</v>
@@ -13702,7 +13704,7 @@
         <v>1428627853.54214</v>
       </c>
       <c r="J216">
-        <v>1571.94855806665</v>
+        <v>1571</v>
       </c>
       <c r="K216">
         <v>624591390.590582</v>
@@ -13762,7 +13764,7 @@
         <v>104619799861.406</v>
       </c>
       <c r="J217">
-        <v>89501.9413936812</v>
+        <v>89501</v>
       </c>
       <c r="K217">
         <v>56457788625.3757</v>
@@ -13822,7 +13824,7 @@
         <v>22587073934.0216</v>
       </c>
       <c r="J218">
-        <v>13369.7974394194</v>
+        <v>13369</v>
       </c>
       <c r="K218">
         <v>21322851842.7245</v>
@@ -13882,7 +13884,7 @@
         <v>125797187783.416</v>
       </c>
       <c r="J219">
-        <v>143852.898333222</v>
+        <v>143852</v>
       </c>
       <c r="K219">
         <v>26916554648.8275</v>
@@ -13942,7 +13944,7 @@
         <v>105014752604.483</v>
       </c>
       <c r="J220">
-        <v>78187.6775408895</v>
+        <v>78187</v>
       </c>
       <c r="K220">
         <v>43014491662.711</v>
@@ -14002,7 +14004,7 @@
         <v>14266708407.9769</v>
       </c>
       <c r="J221">
-        <v>31447.1256730981</v>
+        <v>31447</v>
       </c>
       <c r="K221">
         <v>1968138948.63668</v>
@@ -14062,7 +14064,7 @@
         <v>16822284063.3126</v>
       </c>
       <c r="J222">
-        <v>9533.48203312003</v>
+        <v>9533</v>
       </c>
       <c r="K222">
         <v>1670538017.57674</v>
@@ -14122,7 +14124,7 @@
         <v>75521847167.5862</v>
       </c>
       <c r="J223">
-        <v>112495.512976954</v>
+        <v>112495</v>
       </c>
       <c r="K223">
         <v>27363583780.91</v>
@@ -14182,7 +14184,7 @@
         <v>25643311376.5516</v>
       </c>
       <c r="J224">
-        <v>50602.5223744798</v>
+        <v>50602</v>
       </c>
       <c r="K224">
         <v>2244788851.72259</v>
@@ -14242,7 +14244,7 @@
         <v>101597518322.639</v>
       </c>
       <c r="J225">
-        <v>103987.217304682</v>
+        <v>103987</v>
       </c>
       <c r="K225">
         <v>5575119041.62995</v>
@@ -14302,7 +14304,7 @@
         <v>19027332503.6544</v>
       </c>
       <c r="J226">
-        <v>29574.5732599438</v>
+        <v>29574</v>
       </c>
       <c r="K226">
         <v>2683415915.25328</v>
@@ -14362,7 +14364,7 @@
         <v>1650327892.11249</v>
       </c>
       <c r="J227">
-        <v>1787.13497273982</v>
+        <v>1787</v>
       </c>
       <c r="K227">
         <v>945749518.701748</v>
@@ -14422,7 +14424,7 @@
         <v>112924265631.887</v>
       </c>
       <c r="J228">
-        <v>90863.9271580213</v>
+        <v>90863</v>
       </c>
       <c r="K228">
         <v>43801057524.489</v>
@@ -14482,7 +14484,7 @@
         <v>24101159942.3432</v>
       </c>
       <c r="J229">
-        <v>13655.3577492478</v>
+        <v>13655</v>
       </c>
       <c r="K229">
         <v>20334589907.4134</v>
@@ -14542,7 +14544,7 @@
         <v>137831727239.181</v>
       </c>
       <c r="J230">
-        <v>147391.982662768</v>
+        <v>147391</v>
       </c>
       <c r="K230">
         <v>28315611990.5763</v>
@@ -14602,7 +14604,7 @@
         <v>118919170697.559</v>
       </c>
       <c r="J231">
-        <v>80032.5357969409</v>
+        <v>80032</v>
       </c>
       <c r="K231">
         <v>41019033321.6838</v>
@@ -14662,7 +14664,7 @@
         <v>15449684492.3829</v>
       </c>
       <c r="J232">
-        <v>33707.1853027115</v>
+        <v>33707</v>
       </c>
       <c r="K232">
         <v>1816611590.66081</v>
@@ -14722,7 +14724,7 @@
         <v>19118558566.1344</v>
       </c>
       <c r="J233">
-        <v>9483.21988566801</v>
+        <v>9483</v>
       </c>
       <c r="K233">
         <v>2296312368.76879</v>
@@ -14782,7 +14784,7 @@
         <v>83137177739.9317</v>
       </c>
       <c r="J234">
-        <v>115158.636778068</v>
+        <v>115158</v>
       </c>
       <c r="K234">
         <v>17163517802.4198</v>
@@ -14842,7 +14844,7 @@
         <v>30681074010.4066</v>
       </c>
       <c r="J235">
-        <v>53909.7554524851</v>
+        <v>53909</v>
       </c>
       <c r="K235">
         <v>2524298179.94954</v>
@@ -14902,7 +14904,7 @@
         <v>107092843816.163</v>
       </c>
       <c r="J236">
-        <v>102694.317147385</v>
+        <v>102694</v>
       </c>
       <c r="K236">
         <v>6341537017.67423</v>
@@ -14962,7 +14964,7 @@
         <v>21440304276.0302</v>
       </c>
       <c r="J237">
-        <v>31926.3471830054</v>
+        <v>31926</v>
       </c>
       <c r="K237">
         <v>2879343254.168</v>
@@ -15451,7 +15453,7 @@
         <v>13982311018.7924</v>
       </c>
       <c r="J7">
-        <v>63928.8527653802</v>
+        <v>63928</v>
       </c>
       <c r="K7">
         <v>6516136919.59274</v>
@@ -15515,7 +15517,7 @@
         <v>19975832217.4233</v>
       </c>
       <c r="J8">
-        <v>100576.012248596</v>
+        <v>100576</v>
       </c>
       <c r="K8">
         <v>17359289524.5189</v>
@@ -15579,7 +15581,7 @@
         <v>24291156273.8742</v>
       </c>
       <c r="J9">
-        <v>103902.68580704</v>
+        <v>103902</v>
       </c>
       <c r="K9">
         <v>17442926160.2144</v>
@@ -15643,7 +15645,7 @@
         <v>29743370612.9925</v>
       </c>
       <c r="J10">
-        <v>104036.647790835</v>
+        <v>104036</v>
       </c>
       <c r="K10">
         <v>7961085386.42427</v>
@@ -15707,7 +15709,7 @@
         <v>34131850283.3496</v>
       </c>
       <c r="J11">
-        <v>112274.193929867</v>
+        <v>112274</v>
       </c>
       <c r="K11">
         <v>10581328732.3151</v>
@@ -15771,7 +15773,7 @@
         <v>38240756792.5859</v>
       </c>
       <c r="J12">
-        <v>109399.623065035</v>
+        <v>109399</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -15841,7 +15843,7 @@
         <v>43787874689.4251</v>
       </c>
       <c r="J13">
-        <v>110138.749533575</v>
+        <v>110138</v>
       </c>
       <c r="K13">
         <v>17144628448.139</v>
@@ -15905,7 +15907,7 @@
         <v>50186679222.5088</v>
       </c>
       <c r="J14">
-        <v>109797.749814658</v>
+        <v>109797</v>
       </c>
       <c r="K14">
         <v>28790672811.2985</v>
@@ -15969,7 +15971,7 @@
         <v>56837646365.6924</v>
       </c>
       <c r="J15">
-        <v>107700.426949954</v>
+        <v>107700</v>
       </c>
       <c r="K15">
         <v>78176629453.8231</v>
@@ -16033,7 +16035,7 @@
         <v>61103872632.9691</v>
       </c>
       <c r="J16">
-        <v>103791.208900956</v>
+        <v>103791</v>
       </c>
       <c r="K16">
         <v>26806672376.5168</v>
@@ -16097,7 +16099,7 @@
         <v>65854041864.7401</v>
       </c>
       <c r="J17">
-        <v>100240.446716766</v>
+        <v>100240</v>
       </c>
       <c r="K17">
         <v>17409371770.145</v>
@@ -16157,7 +16159,7 @@
         <v>70584977309.7717</v>
       </c>
       <c r="J18">
-        <v>97466.9972261083</v>
+        <v>97466</v>
       </c>
       <c r="K18">
         <v>17036239960.98</v>
@@ -16217,7 +16219,7 @@
         <v>76120684622.3108</v>
       </c>
       <c r="J19">
-        <v>94566.085657076</v>
+        <v>94566</v>
       </c>
       <c r="K19">
         <v>21403883661.2124</v>
@@ -16337,7 +16339,7 @@
         <v>78278216489.3034</v>
       </c>
       <c r="J21">
-        <v>84764.4647407208</v>
+        <v>84764</v>
       </c>
       <c r="K21">
         <v>40941559983.9069</v>
@@ -16397,7 +16399,7 @@
         <v>84122098877.8656</v>
       </c>
       <c r="J22">
-        <v>86333.0943782653</v>
+        <v>86333</v>
       </c>
       <c r="K22">
         <v>83942983585.5647</v>
@@ -16457,7 +16459,7 @@
         <v>95609914033.8778</v>
       </c>
       <c r="J23">
-        <v>89467.5060887856</v>
+        <v>89467</v>
       </c>
       <c r="K23">
         <v>69687013752.2493</v>
@@ -16517,7 +16519,7 @@
         <v>104619799861.406</v>
       </c>
       <c r="J24">
-        <v>89501.9413936812</v>
+        <v>89501</v>
       </c>
       <c r="K24">
         <v>56457788625.3757</v>
@@ -16577,7 +16579,7 @@
         <v>112924265631.887</v>
       </c>
       <c r="J25">
-        <v>90863.9271580213</v>
+        <v>90863</v>
       </c>
       <c r="K25">
         <v>43801057524.489</v>
@@ -16730,13 +16732,13 @@
         <v>2006</v>
       </c>
       <c r="B7">
-        <v>0.291924152221065</v>
+        <v>0.291924152221064</v>
       </c>
       <c r="C7">
-        <v>131022070046.052</v>
+        <v>131022070046.053</v>
       </c>
       <c r="D7">
-        <v>0.258847666940384</v>
+        <v>0.258847666940383</v>
       </c>
       <c r="E7">
         <v>1.05865039128914</v>
@@ -16767,7 +16769,7 @@
         <v>0.28173131463118</v>
       </c>
       <c r="C9">
-        <v>204703481976.649</v>
+        <v>204703481976.648</v>
       </c>
       <c r="D9">
         <v>0.302534403617726</v>
@@ -16781,13 +16783,13 @@
         <v>2009</v>
       </c>
       <c r="B10">
-        <v>0.29821128576218</v>
+        <v>0.298211285762181</v>
       </c>
       <c r="C10">
         <v>184112276048.956</v>
       </c>
       <c r="D10">
-        <v>0.380180414908556</v>
+        <v>0.380180414908557</v>
       </c>
       <c r="E10">
         <v>1.19118368851591</v>
@@ -16801,7 +16803,7 @@
         <v>0.320024753285429</v>
       </c>
       <c r="C11">
-        <v>203050594183.492</v>
+        <v>203050594183.493</v>
       </c>
       <c r="D11">
         <v>0.357161879014824</v>
@@ -16818,7 +16820,7 @@
         <v>0.30275953361088</v>
       </c>
       <c r="C12">
-        <v>225013520538.727</v>
+        <v>225013520538.726</v>
       </c>
       <c r="D12">
         <v>0.39138359763031</v>
@@ -16851,13 +16853,13 @@
         <v>2013</v>
       </c>
       <c r="B14">
-        <v>0.284364147665339</v>
+        <v>0.284364147665338</v>
       </c>
       <c r="C14">
-        <v>281599544926.558</v>
+        <v>281599544926.559</v>
       </c>
       <c r="D14">
-        <v>0.4485116840801</v>
+        <v>0.448511684080101</v>
       </c>
       <c r="E14">
         <v>1.16450299425308</v>
@@ -16902,7 +16904,7 @@
         <v>2016</v>
       </c>
       <c r="B17">
-        <v>0.318223007298673</v>
+        <v>0.318223007298674</v>
       </c>
       <c r="C17">
         <v>332900017802.479</v>
@@ -16919,10 +16921,10 @@
         <v>2017</v>
       </c>
       <c r="B18">
-        <v>0.339620881998154</v>
+        <v>0.339620881998153</v>
       </c>
       <c r="C18">
-        <v>319716953542.574</v>
+        <v>319716953542.575</v>
       </c>
       <c r="D18">
         <v>0.429284847789789</v>
@@ -16936,13 +16938,13 @@
         <v>2018</v>
       </c>
       <c r="B19">
-        <v>0.347144803240304</v>
+        <v>0.347144803240303</v>
       </c>
       <c r="C19">
         <v>372151519563.687</v>
       </c>
       <c r="D19">
-        <v>0.38467068091003</v>
+        <v>0.384670680910031</v>
       </c>
       <c r="E19">
         <v>1.16706303143822</v>
@@ -16976,7 +16978,7 @@
         <v>417854417660.489</v>
       </c>
       <c r="D21">
-        <v>0.427836060376059</v>
+        <v>0.427836060376058</v>
       </c>
       <c r="E21">
         <v>1.61957565994111</v>
@@ -17027,7 +17029,7 @@
         <v>569465342893.417</v>
       </c>
       <c r="D24">
-        <v>0.435684992767357</v>
+        <v>0.435684992767355</v>
       </c>
       <c r="E24">
         <v>1.67604027971978</v>
@@ -17044,10 +17046,2119 @@
         <v>594101282305.454</v>
       </c>
       <c r="D25">
-        <v>0.427791515927841</v>
+        <v>0.42779151592784</v>
       </c>
       <c r="E25">
         <v>1.65536015099205</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>anno</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>seccion</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>epoca</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ciiu_version</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>vbp_pp</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>vbp_pb</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>vab_pp</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>vab_pb</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>remuneraciones</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>puestos_trabajo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>fbcf</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>adquisiciones_importadas</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>consumo_capital</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>impuestos_netos</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>stock_capital</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>excedente_bruto</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>part_salarial</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>productividad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>2001</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Rev.3</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>224795374000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2">
+        <v>105965497000</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I2">
+        <v>48921033000</v>
+      </c>
+      <c r="J2">
+        <v>538624</v>
+      </c>
+      <c r="K2">
+        <v>15584526000</v>
+      </c>
+      <c r="L2">
+        <v>3176411000</v>
+      </c>
+      <c r="M2">
+        <v>9474344000</v>
+      </c>
+      <c r="N2">
+        <v>8228656000</v>
+      </c>
+      <c r="O2">
+        <v>123851491000</v>
+      </c>
+      <c r="P2">
+        <v>57044464000</v>
+      </c>
+      <c r="Q2">
+        <v>0.461669452652121</v>
+      </c>
+      <c r="R2">
+        <v>196733.708486811</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2002</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Rev.3</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>228293239248</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3">
+        <v>106353797467</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I3">
+        <v>42622839206</v>
+      </c>
+      <c r="J3">
+        <v>339997</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M3">
+        <v>11163880916</v>
+      </c>
+      <c r="N3">
+        <v>7193975850</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P3">
+        <v>63730958261</v>
+      </c>
+      <c r="Q3">
+        <v>0.400764619798604</v>
+      </c>
+      <c r="R3">
+        <v>312808.046738648</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>2003</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Rev.3</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>282760554719</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4">
+        <v>117480701268</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I4">
+        <v>44485282167</v>
+      </c>
+      <c r="J4">
+        <v>345219</v>
+      </c>
+      <c r="K4">
+        <v>14939026955</v>
+      </c>
+      <c r="L4">
+        <v>5765671714</v>
+      </c>
+      <c r="M4">
+        <v>15388019830</v>
+      </c>
+      <c r="N4">
+        <v>7667299026</v>
+      </c>
+      <c r="O4">
+        <v>128858476811</v>
+      </c>
+      <c r="P4">
+        <v>72995419101</v>
+      </c>
+      <c r="Q4">
+        <v>0.378660338990649</v>
+      </c>
+      <c r="R4">
+        <v>340307.750349778</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2004</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Rev.3</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>342486970874</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G5">
+        <v>137248675768</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I5">
+        <v>48007488282</v>
+      </c>
+      <c r="J5">
+        <v>348339</v>
+      </c>
+      <c r="K5">
+        <v>20956681133</v>
+      </c>
+      <c r="L5">
+        <v>2372629177</v>
+      </c>
+      <c r="M5">
+        <v>17341745740</v>
+      </c>
+      <c r="N5">
+        <v>8870370869</v>
+      </c>
+      <c r="O5">
+        <v>187339221901</v>
+      </c>
+      <c r="P5">
+        <v>89241187486</v>
+      </c>
+      <c r="Q5">
+        <v>0.349784710222997</v>
+      </c>
+      <c r="R5">
+        <v>394008.927418406</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>2005</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rev.3</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>370267989847</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G6">
+        <v>152188634950</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6">
+        <v>56739334938</v>
+      </c>
+      <c r="J6">
+        <v>391484</v>
+      </c>
+      <c r="K6">
+        <v>22308747111</v>
+      </c>
+      <c r="L6">
+        <v>3786737908</v>
+      </c>
+      <c r="M6">
+        <v>17296133580</v>
+      </c>
+      <c r="N6">
+        <v>9812890558</v>
+      </c>
+      <c r="O6">
+        <v>239076254150</v>
+      </c>
+      <c r="P6">
+        <v>95449300012</v>
+      </c>
+      <c r="Q6">
+        <v>0.372822418419359</v>
+      </c>
+      <c r="R6">
+        <v>388748.032997517</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>2006</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Rev.3</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>336442815360.939</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G7">
+        <v>131310154037.695</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I7">
+        <v>47362257399.2046</v>
+      </c>
+      <c r="J7">
+        <v>205950</v>
+      </c>
+      <c r="K7">
+        <v>19150720336.4055</v>
+      </c>
+      <c r="L7">
+        <v>3231971966.12888</v>
+      </c>
+      <c r="M7">
+        <v>131310154037.695</v>
+      </c>
+      <c r="N7">
+        <v>17116477319.5601</v>
+      </c>
+      <c r="O7">
+        <v>231687199104.872</v>
+      </c>
+      <c r="P7">
+        <v>83947896638.4905</v>
+      </c>
+      <c r="Q7">
+        <v>0.360689984306989</v>
+      </c>
+      <c r="R7">
+        <v>637582.685300777</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>2007</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Rev.3</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>481369119712.772</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8">
+        <v>196898700963.264</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8">
+        <v>75965597899.6002</v>
+      </c>
+      <c r="J8">
+        <v>384435</v>
+      </c>
+      <c r="K8">
+        <v>38859260194.9979</v>
+      </c>
+      <c r="L8">
+        <v>4047231987.45161</v>
+      </c>
+      <c r="M8">
+        <v>196898700963.264</v>
+      </c>
+      <c r="N8">
+        <v>21950974301.9375</v>
+      </c>
+      <c r="O8">
+        <v>291955588783.621</v>
+      </c>
+      <c r="P8">
+        <v>120933103063.664</v>
+      </c>
+      <c r="Q8">
+        <v>0.385810559074096</v>
+      </c>
+      <c r="R8">
+        <v>512176.83343937</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>2008</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>559144297146.625</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G9">
+        <v>205890238511.316</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I9">
+        <v>94216384323.7464</v>
+      </c>
+      <c r="J9">
+        <v>436440</v>
+      </c>
+      <c r="K9">
+        <v>43310215637.4511</v>
+      </c>
+      <c r="L9">
+        <v>9013827403.17803</v>
+      </c>
+      <c r="M9">
+        <v>25276649939.0697</v>
+      </c>
+      <c r="N9">
+        <v>8127087389.63337</v>
+      </c>
+      <c r="O9">
+        <v>333451079195.265</v>
+      </c>
+      <c r="P9">
+        <v>111673854187.57</v>
+      </c>
+      <c r="Q9">
+        <v>0.457604911262308</v>
+      </c>
+      <c r="R9">
+        <v>471749.240471351</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>2009</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E10">
+        <v>572525294843.88</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G10">
+        <v>234652404427.536</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10">
+        <v>117108913106.686</v>
+      </c>
+      <c r="J10">
+        <v>477456</v>
+      </c>
+      <c r="K10">
+        <v>37495334384.0992</v>
+      </c>
+      <c r="L10">
+        <v>9679386069.55089</v>
+      </c>
+      <c r="M10">
+        <v>26688200109.4006</v>
+      </c>
+      <c r="N10">
+        <v>8225554423.77405</v>
+      </c>
+      <c r="O10">
+        <v>346393993604.053</v>
+      </c>
+      <c r="P10">
+        <v>117543491320.85</v>
+      </c>
+      <c r="Q10">
+        <v>0.499073995821129</v>
+      </c>
+      <c r="R10">
+        <v>491463.934744849</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>2010</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E11">
+        <v>709424887808.739</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G11">
+        <v>308305260093.789</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I11">
+        <v>144685743750.673</v>
+      </c>
+      <c r="J11">
+        <v>522280</v>
+      </c>
+      <c r="K11">
+        <v>61076798987.5527</v>
+      </c>
+      <c r="L11">
+        <v>9345396138.26938</v>
+      </c>
+      <c r="M11">
+        <v>31780276848.6609</v>
+      </c>
+      <c r="N11">
+        <v>11905200627.3829</v>
+      </c>
+      <c r="O11">
+        <v>449096205806.534</v>
+      </c>
+      <c r="P11">
+        <v>163619516343.116</v>
+      </c>
+      <c r="Q11">
+        <v>0.469293789235572</v>
+      </c>
+      <c r="R11">
+        <v>590306.464145265</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>2011</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E12">
+        <v>771498581508.335</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G12">
+        <v>329709117763.868</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I12">
+        <v>172970589361.342</v>
+      </c>
+      <c r="J12">
+        <v>542453</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M12">
+        <v>172970589361.342</v>
+      </c>
+      <c r="N12">
+        <v>329709117763.868</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P12">
+        <v>156738528402.527</v>
+      </c>
+      <c r="Q12">
+        <v>0.524615729569299</v>
+      </c>
+      <c r="R12">
+        <v>607811.40073678</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>2012</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E13">
+        <v>908716083147.998</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G13">
+        <v>380803978320.661</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I13">
+        <v>204379867609.763</v>
+      </c>
+      <c r="J13">
+        <v>564838</v>
+      </c>
+      <c r="K13">
+        <v>70402576883.8423</v>
+      </c>
+      <c r="L13">
+        <v>16418462867.3078</v>
+      </c>
+      <c r="M13">
+        <v>35113806680.2514</v>
+      </c>
+      <c r="N13">
+        <v>19479252420.6849</v>
+      </c>
+      <c r="O13">
+        <v>490287039450.532</v>
+      </c>
+      <c r="P13">
+        <v>176424110710.899</v>
+      </c>
+      <c r="Q13">
+        <v>0.536706230095269</v>
+      </c>
+      <c r="R13">
+        <v>674182.64762757</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>2013</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E14">
+        <v>1029630572140.08</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G14">
+        <v>446438532539.492</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I14">
+        <v>239717322965.669</v>
+      </c>
+      <c r="J14">
+        <v>592292</v>
+      </c>
+      <c r="K14">
+        <v>95632259933.4402</v>
+      </c>
+      <c r="L14">
+        <v>14065686833.8348</v>
+      </c>
+      <c r="M14">
+        <v>37001352296.9516</v>
+      </c>
+      <c r="N14">
+        <v>24693359137.995</v>
+      </c>
+      <c r="O14">
+        <v>551876752379.702</v>
+      </c>
+      <c r="P14">
+        <v>206721209573.824</v>
+      </c>
+      <c r="Q14">
+        <v>0.536954822430035</v>
+      </c>
+      <c r="R14">
+        <v>753747.362009773</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>2014</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E15">
+        <v>1199313983186.27</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G15">
+        <v>525321848898.882</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I15">
+        <v>280926635663.202</v>
+      </c>
+      <c r="J15">
+        <v>616854</v>
+      </c>
+      <c r="K15">
+        <v>159227973748.991</v>
+      </c>
+      <c r="L15">
+        <v>16710161650.4979</v>
+      </c>
+      <c r="M15">
+        <v>44318807852.1372</v>
+      </c>
+      <c r="N15">
+        <v>26736846637.0949</v>
+      </c>
+      <c r="O15">
+        <v>676414498513.775</v>
+      </c>
+      <c r="P15">
+        <v>244395213235.68</v>
+      </c>
+      <c r="Q15">
+        <v>0.534770514974862</v>
+      </c>
+      <c r="R15">
+        <v>851614.561790768</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>2015</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E16">
+        <v>1338814807883.4</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G16">
+        <v>607207545851.913</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I16">
+        <v>318079975456.983</v>
+      </c>
+      <c r="J16">
+        <v>618974</v>
+      </c>
+      <c r="K16">
+        <v>105224852365.573</v>
+      </c>
+      <c r="L16">
+        <v>12495622149.4769</v>
+      </c>
+      <c r="M16">
+        <v>53390559582.1431</v>
+      </c>
+      <c r="N16">
+        <v>35268317264.4714</v>
+      </c>
+      <c r="O16">
+        <v>736061470775.725</v>
+      </c>
+      <c r="P16">
+        <v>289127570394.93</v>
+      </c>
+      <c r="Q16">
+        <v>0.523840616984949</v>
+      </c>
+      <c r="R16">
+        <v>980990.390310277</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>2016</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E17">
+        <v>1402607775102.32</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G17">
+        <v>651676760423.003</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I17">
+        <v>350937641730.853</v>
+      </c>
+      <c r="J17">
+        <v>614478</v>
+      </c>
+      <c r="K17">
+        <v>103984369912.072</v>
+      </c>
+      <c r="L17">
+        <v>9730133740.5832</v>
+      </c>
+      <c r="M17">
+        <v>54852592008.4201</v>
+      </c>
+      <c r="N17">
+        <v>40295879959.7307</v>
+      </c>
+      <c r="O17">
+        <v>806021467568.495</v>
+      </c>
+      <c r="P17">
+        <v>300739118692.15</v>
+      </c>
+      <c r="Q17">
+        <v>0.538514894259938</v>
+      </c>
+      <c r="R17">
+        <v>1060537.17207614</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>2017</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E18">
+        <v>1487902627065.02</v>
+      </c>
+      <c r="F18">
+        <v>1443196189138.68</v>
+      </c>
+      <c r="G18">
+        <v>718899634453.725</v>
+      </c>
+      <c r="H18">
+        <v>674193196527.387</v>
+      </c>
+      <c r="I18">
+        <v>385131881530.737</v>
+      </c>
+      <c r="J18">
+        <v>619820</v>
+      </c>
+      <c r="K18">
+        <v>95576488801.99</v>
+      </c>
+      <c r="L18">
+        <v>10298175130.96</v>
+      </c>
+      <c r="M18">
+        <v>60215993660.88</v>
+      </c>
+      <c r="N18">
+        <v>1762120524.19</v>
+      </c>
+      <c r="O18">
+        <v>841966030516.03</v>
+      </c>
+      <c r="P18">
+        <v>333767752922.988</v>
+      </c>
+      <c r="Q18">
+        <v>0.53572413042523</v>
+      </c>
+      <c r="R18">
+        <v>1159852.2707459</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>2018</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E19">
+        <v>1658683685335.02</v>
+      </c>
+      <c r="F19">
+        <v>1614155725631.5</v>
+      </c>
+      <c r="G19">
+        <v>789921510187.459</v>
+      </c>
+      <c r="H19">
+        <v>745393550483.945</v>
+      </c>
+      <c r="I19">
+        <v>422590435418.063</v>
+      </c>
+      <c r="J19">
+        <v>620089</v>
+      </c>
+      <c r="K19">
+        <v>97638209970.69</v>
+      </c>
+      <c r="L19">
+        <v>12591274268.9296</v>
+      </c>
+      <c r="M19">
+        <v>62139743088.513</v>
+      </c>
+      <c r="N19">
+        <v>2249888267.33789</v>
+      </c>
+      <c r="O19">
+        <v>898330263751.352</v>
+      </c>
+      <c r="P19">
+        <v>367331074769.396</v>
+      </c>
+      <c r="Q19">
+        <v>0.534977754078094</v>
+      </c>
+      <c r="R19">
+        <v>1273884.08790909</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>2019</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E20">
+        <v>1790503155926</v>
+      </c>
+      <c r="F20">
+        <v>1742328722361</v>
+      </c>
+      <c r="G20">
+        <v>824315284444</v>
+      </c>
+      <c r="H20">
+        <v>776140850879</v>
+      </c>
+      <c r="I20">
+        <v>456264699852</v>
+      </c>
+      <c r="J20">
+        <v>611937</v>
+      </c>
+      <c r="K20">
+        <v>128886507624</v>
+      </c>
+      <c r="L20">
+        <v>16497801681</v>
+      </c>
+      <c r="M20">
+        <v>68724454704.9513</v>
+      </c>
+      <c r="N20">
+        <v>3512792203.01998</v>
+      </c>
+      <c r="O20">
+        <v>995997166119</v>
+      </c>
+      <c r="P20">
+        <v>368050584592</v>
+      </c>
+      <c r="Q20">
+        <v>0.553507509156221</v>
+      </c>
+      <c r="R20">
+        <v>1347059.06726346</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>2020</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E21">
+        <v>1805094127854.9</v>
+      </c>
+      <c r="F21">
+        <v>1752134676072.14</v>
+      </c>
+      <c r="G21">
+        <v>838326089885.307</v>
+      </c>
+      <c r="H21">
+        <v>785366638102.545</v>
+      </c>
+      <c r="I21">
+        <v>445768537897.996</v>
+      </c>
+      <c r="J21">
+        <v>570243</v>
+      </c>
+      <c r="K21">
+        <v>116968594615.136</v>
+      </c>
+      <c r="L21">
+        <v>11107721184.8042</v>
+      </c>
+      <c r="M21">
+        <v>72470063542.389</v>
+      </c>
+      <c r="N21">
+        <v>23526226.0532918</v>
+      </c>
+      <c r="O21">
+        <v>1042958318864.71</v>
+      </c>
+      <c r="P21">
+        <v>392557551987.311</v>
+      </c>
+      <c r="Q21">
+        <v>0.531736448711721</v>
+      </c>
+      <c r="R21">
+        <v>1470120.79040919</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>2021</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E22">
+        <v>2173653003453.79</v>
+      </c>
+      <c r="F22">
+        <v>2156399403913.47</v>
+      </c>
+      <c r="G22">
+        <v>1016152775933.43</v>
+      </c>
+      <c r="H22">
+        <v>998899176393.096</v>
+      </c>
+      <c r="I22">
+        <v>470199821189.107</v>
+      </c>
+      <c r="J22">
+        <v>602971</v>
+      </c>
+      <c r="K22">
+        <v>187321533925.961</v>
+      </c>
+      <c r="L22">
+        <v>19537003773.2717</v>
+      </c>
+      <c r="M22">
+        <v>73799557031.8412</v>
+      </c>
+      <c r="N22">
+        <v>-429188905.676115</v>
+      </c>
+      <c r="O22">
+        <v>1173390818677.98</v>
+      </c>
+      <c r="P22">
+        <v>545952954744.318</v>
+      </c>
+      <c r="Q22">
+        <v>0.462725519553089</v>
+      </c>
+      <c r="R22">
+        <v>1685243.19732363</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>2022</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E23">
+        <v>2441897021618.8</v>
+      </c>
+      <c r="F23">
+        <v>2395110854824.29</v>
+      </c>
+      <c r="G23">
+        <v>1082579648621.82</v>
+      </c>
+      <c r="H23">
+        <v>1035793481827.32</v>
+      </c>
+      <c r="I23">
+        <v>522254664756.318</v>
+      </c>
+      <c r="J23">
+        <v>627082</v>
+      </c>
+      <c r="K23">
+        <v>183033331632.185</v>
+      </c>
+      <c r="L23">
+        <v>17797191552.4107</v>
+      </c>
+      <c r="M23">
+        <v>74486121315.7251</v>
+      </c>
+      <c r="N23">
+        <v>-2575703321.18187</v>
+      </c>
+      <c r="O23">
+        <v>1205661045725.29</v>
+      </c>
+      <c r="P23">
+        <v>560324983865.504</v>
+      </c>
+      <c r="Q23">
+        <v>0.4824168507335</v>
+      </c>
+      <c r="R23">
+        <v>1726376.53229055</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>2023</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E24">
+        <v>2518876758620.81</v>
+      </c>
+      <c r="F24">
+        <v>2469821836459.87</v>
+      </c>
+      <c r="G24">
+        <v>1143758788706.06</v>
+      </c>
+      <c r="H24">
+        <v>1094703866545.12</v>
+      </c>
+      <c r="I24">
+        <v>612326443878.589</v>
+      </c>
+      <c r="J24">
+        <v>664118</v>
+      </c>
+      <c r="K24">
+        <v>189841862725.959</v>
+      </c>
+      <c r="L24">
+        <v>15278811501.6459</v>
+      </c>
+      <c r="M24">
+        <v>85762171452.3847</v>
+      </c>
+      <c r="N24">
+        <v>-221349059.58439</v>
+      </c>
+      <c r="O24">
+        <v>1284742421782.95</v>
+      </c>
+      <c r="P24">
+        <v>531432344827.468</v>
+      </c>
+      <c r="Q24">
+        <v>0.535363268833386</v>
+      </c>
+      <c r="R24">
+        <v>1722222.23867755</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>2024</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>economia_total</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Rev.4</t>
+        </is>
+      </c>
+      <c r="E25">
+        <v>2723572147079.9</v>
+      </c>
+      <c r="F25">
+        <v>2670777146626.85</v>
+      </c>
+      <c r="G25">
+        <v>1257042954849.99</v>
+      </c>
+      <c r="H25">
+        <v>1204247954396.94</v>
+      </c>
+      <c r="I25">
+        <v>672346294304.131</v>
+      </c>
+      <c r="J25">
+        <v>680605</v>
+      </c>
+      <c r="K25">
+        <v>167437662476.505</v>
+      </c>
+      <c r="L25">
+        <v>15575384069.883</v>
+      </c>
+      <c r="M25">
+        <v>92718688124.5785</v>
+      </c>
+      <c r="N25">
+        <v>274718190.319679</v>
+      </c>
+      <c r="O25">
+        <v>1395438696039.73</v>
+      </c>
+      <c r="P25">
+        <v>584696660545.855</v>
+      </c>
+      <c r="Q25">
+        <v>0.534863420307199</v>
+      </c>
+      <c r="R25">
+        <v>1846949.33897045</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>anno</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>vab_vbp</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>consumo_intermedio_vbp_menos_vab</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>remuneraciones_vab</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stock_vab</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>2001</v>
+      </c>
+      <c r="B2">
+        <v>0.471386466342497</v>
+      </c>
+      <c r="C2">
+        <v>118829877000</v>
+      </c>
+      <c r="D2">
+        <v>0.461669452652121</v>
+      </c>
+      <c r="E2">
+        <v>1.16879073383669</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2002</v>
+      </c>
+      <c r="B3">
+        <v>0.465864857922777</v>
+      </c>
+      <c r="C3">
+        <v>121939441781</v>
+      </c>
+      <c r="D3">
+        <v>0.400764619798604</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>2003</v>
+      </c>
+      <c r="B4">
+        <v>0.415477687065472</v>
+      </c>
+      <c r="C4">
+        <v>165279853451</v>
+      </c>
+      <c r="D4">
+        <v>0.378660338990649</v>
+      </c>
+      <c r="E4">
+        <v>1.09684803904128</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2004</v>
+      </c>
+      <c r="B5">
+        <v>0.400741305334192</v>
+      </c>
+      <c r="C5">
+        <v>205238295106</v>
+      </c>
+      <c r="D5">
+        <v>0.349784710222997</v>
+      </c>
+      <c r="E5">
+        <v>1.36496196304051</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>2005</v>
+      </c>
+      <c r="B6">
+        <v>0.41102293237092</v>
+      </c>
+      <c r="C6">
+        <v>218079354897</v>
+      </c>
+      <c r="D6">
+        <v>0.372822418419359</v>
+      </c>
+      <c r="E6">
+        <v>1.57092055020105</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>2006</v>
+      </c>
+      <c r="B7">
+        <v>0.390289666007058</v>
+      </c>
+      <c r="C7">
+        <v>205132661323.244</v>
+      </c>
+      <c r="D7">
+        <v>0.360689984306989</v>
+      </c>
+      <c r="E7">
+        <v>1.76442713667339</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>2007</v>
+      </c>
+      <c r="B8">
+        <v>0.409038911928442</v>
+      </c>
+      <c r="C8">
+        <v>284470418749.508</v>
+      </c>
+      <c r="D8">
+        <v>0.385810559074096</v>
+      </c>
+      <c r="E8">
+        <v>1.48277051781104</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>2008</v>
+      </c>
+      <c r="B9">
+        <v>0.368223801194069</v>
+      </c>
+      <c r="C9">
+        <v>353254058635.309</v>
+      </c>
+      <c r="D9">
+        <v>0.457604911262308</v>
+      </c>
+      <c r="E9">
+        <v>1.61955749629644</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>2009</v>
+      </c>
+      <c r="B10">
+        <v>0.409855086824632</v>
+      </c>
+      <c r="C10">
+        <v>337872890416.344</v>
+      </c>
+      <c r="D10">
+        <v>0.499073995821129</v>
+      </c>
+      <c r="E10">
+        <v>1.47620048662669</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>2010</v>
+      </c>
+      <c r="B11">
+        <v>0.434584781830925</v>
+      </c>
+      <c r="C11">
+        <v>401119627714.95</v>
+      </c>
+      <c r="D11">
+        <v>0.469293789235572</v>
+      </c>
+      <c r="E11">
+        <v>1.45666086160812</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>2011</v>
+      </c>
+      <c r="B12">
+        <v>0.427361923490855</v>
+      </c>
+      <c r="C12">
+        <v>441789463744.466</v>
+      </c>
+      <c r="D12">
+        <v>0.524615729569299</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>2012</v>
+      </c>
+      <c r="B13">
+        <v>0.419057156996133</v>
+      </c>
+      <c r="C13">
+        <v>527912104827.337</v>
+      </c>
+      <c r="D13">
+        <v>0.536706230095269</v>
+      </c>
+      <c r="E13">
+        <v>1.28750503503847</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>2013</v>
+      </c>
+      <c r="B14">
+        <v>0.43359098362005</v>
+      </c>
+      <c r="C14">
+        <v>583192039600.589</v>
+      </c>
+      <c r="D14">
+        <v>0.536954822430035</v>
+      </c>
+      <c r="E14">
+        <v>1.23617634266568</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>2014</v>
+      </c>
+      <c r="B15">
+        <v>0.438018614194122</v>
+      </c>
+      <c r="C15">
+        <v>673992134287.387</v>
+      </c>
+      <c r="D15">
+        <v>0.534770514974862</v>
+      </c>
+      <c r="E15">
+        <v>1.28761919941384</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>2015</v>
+      </c>
+      <c r="B16">
+        <v>0.453541103875208</v>
+      </c>
+      <c r="C16">
+        <v>731607262031.49</v>
+      </c>
+      <c r="D16">
+        <v>0.523840616984949</v>
+      </c>
+      <c r="E16">
+        <v>1.21220738412107</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>2016</v>
+      </c>
+      <c r="B17">
+        <v>0.464617958057064</v>
+      </c>
+      <c r="C17">
+        <v>750931014679.32</v>
+      </c>
+      <c r="D17">
+        <v>0.538514894259938</v>
+      </c>
+      <c r="E17">
+        <v>1.23684242943589</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>2017</v>
+      </c>
+      <c r="B18">
+        <v>0.483163092380446</v>
+      </c>
+      <c r="C18">
+        <v>769002992611.296</v>
+      </c>
+      <c r="D18">
+        <v>0.53572413042523</v>
+      </c>
+      <c r="E18">
+        <v>1.17118717295749</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>2018</v>
+      </c>
+      <c r="B19">
+        <v>0.476233966229621</v>
+      </c>
+      <c r="C19">
+        <v>868762175147.557</v>
+      </c>
+      <c r="D19">
+        <v>0.534977754078094</v>
+      </c>
+      <c r="E19">
+        <v>1.13723990569413</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>2019</v>
+      </c>
+      <c r="B20">
+        <v>0.460381922095907</v>
+      </c>
+      <c r="C20">
+        <v>966187871482</v>
+      </c>
+      <c r="D20">
+        <v>0.553507509156221</v>
+      </c>
+      <c r="E20">
+        <v>1.20827210766909</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>2020</v>
+      </c>
+      <c r="B21">
+        <v>0.46442236831247</v>
+      </c>
+      <c r="C21">
+        <v>966768037969.596</v>
+      </c>
+      <c r="D21">
+        <v>0.531736448711721</v>
+      </c>
+      <c r="E21">
+        <v>1.24409621917815</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>2021</v>
+      </c>
+      <c r="B22">
+        <v>0.467486196885531</v>
+      </c>
+      <c r="C22">
+        <v>1157500227520.37</v>
+      </c>
+      <c r="D22">
+        <v>0.462725519553089</v>
+      </c>
+      <c r="E22">
+        <v>1.15473858505196</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>2022</v>
+      </c>
+      <c r="B23">
+        <v>0.443335504747924</v>
+      </c>
+      <c r="C23">
+        <v>1359317372996.97</v>
+      </c>
+      <c r="D23">
+        <v>0.4824168507335</v>
+      </c>
+      <c r="E23">
+        <v>1.11369269435293</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>2023</v>
+      </c>
+      <c r="B24">
+        <v>0.454074930340107</v>
+      </c>
+      <c r="C24">
+        <v>1375117969914.75</v>
+      </c>
+      <c r="D24">
+        <v>0.535363268833386</v>
+      </c>
+      <c r="E24">
+        <v>1.12326343147613</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>2024</v>
+      </c>
+      <c r="B25">
+        <v>0.461542006954996</v>
+      </c>
+      <c r="C25">
+        <v>1466529192229.92</v>
+      </c>
+      <c r="D25">
+        <v>0.534863420307199</v>
+      </c>
+      <c r="E25">
+        <v>1.11009627050196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>